<commit_message>
Career mode: bribe system, walk-on volume, new opponent images, UI fixes
- Mad Dog bribe/throw system (L5): throw-a-leg offer + bribe-back at match point
- Walk-on music volume choice: quiet/medium/loud/deafening affects opponent anger
- Lars and Vinnie images wired into opponent_data
- New character images: Steve, Lisa Mad Dog, Manager, Unknown Caller, old lost man
- Tungsten/Premium Tungsten dart colours lightened for visibility against black board
- Coach intro card removed (redundant), "HIRE A COACH" -> "HIRE THE COACH"
- Vinnie intro: "gold teeth" -> "gold tooth"
- Manager silk shirt text: removed deep purple reference, elegantly lifts
- Sponsor rep: removed "fill your shirt out" line
- Walk-on music card: fixed text overflow, added autowrap
- Manager motivational speech: trimmed to fit on screen
- Bling card: "sovereign ring" -> "a bit of gold"
- Career overview docs and spec updates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/career_progression_spec.xlsx
+++ b/docs/career_progression_spec.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Career Journey" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swagger Progression" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2866,4 +2867,198 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Star</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Player Choice</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Shopping Spree</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Forced — companion drags you</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Bling + matching tattoos with your mate. First visible change to appearance.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Already wired in code. £20 spend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>First Celebration</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Pick style: The Flex / The Big Fish / Down a Pint</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>First celebration is automated in-match. Boosts confidence, makes opponent angry. NOT enough for a fight first time.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Down a Pint costs a pint at venue price + adds one drink level. From here on, celebrations available every leg win.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Silk Shirt</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Gift — not optional</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Coach/manager says ‘not having my player looking like that’ and gifts a silk shirt. Look the part for the bigger stages.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Narrative moment. No cost. Triggers at level where coach is active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Dodgy Bet on Yourself</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Choose AMOUNT (not whether)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Place a bet on yourself before the match. Win the match = win the bet = swagger star. The amount is the choice, not the act.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Ties into gambling mechanic from The Contact (L4). Pure ego move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Walk-On Music</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pick your track (3 options)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Choose your entrance music. From this point, every match starts with a walk-on sequence. The ultimate swagger.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>The crowd goes before you’ve even thrown a dart.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>